<commit_message>
Actualización de productos y menú 2026
</commit_message>
<xml_diff>
--- a/public/data/productos.xlsx
+++ b/public/data/productos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
   <si>
     <t xml:space="preserve">Nombre</t>
   </si>
@@ -97,6 +97,15 @@
     <t xml:space="preserve">Hay 5 juegos acá</t>
   </si>
   <si>
+    <t xml:space="preserve">Torta naranja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas10.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lindas mariposas</t>
+  </si>
+  <si>
     <t xml:space="preserve">Torta mamá</t>
   </si>
   <si>
@@ -131,6 +140,60 @@
   </si>
   <si>
     <t xml:space="preserve">Otra más de color rosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta papá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas8.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trae cerveza incluida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta mariposas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas9.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trae mariposas rosadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta osito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas11.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiene un osito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta dulce de leche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas12.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trae bastante dulce de leche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta choco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas13.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puro sabor choco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta duraznos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas14.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiene duraznos buenos</t>
   </si>
 </sst>
 </file>
@@ -341,11 +404,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="57.33"/>
   </cols>
   <sheetData>
@@ -469,11 +533,11 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>2300</v>
+        <v>1900</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>26</v>
@@ -490,7 +554,7 @@
         <v>28</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>3100</v>
+        <v>2300</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>29</v>
@@ -507,13 +571,13 @@
         <v>31</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>690</v>
+        <v>3100</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>33</v>
@@ -524,16 +588,135 @@
         <v>34</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>2400</v>
+        <v>690</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>3400</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>3100</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza productos y componentes UI: mejoras en header, cards, FAQ y agrega ScrollToTop
</commit_message>
<xml_diff>
--- a/public/data/productos.xlsx
+++ b/public/data/productos.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Descripcion</t>
   </si>
   <si>
-    <t xml:space="preserve">Torta rosa</t>
+    <t xml:space="preserve">Torta Princesa</t>
   </si>
   <si>
     <t xml:space="preserve">tortas1.png</t>
@@ -46,16 +46,124 @@
     <t xml:space="preserve">Tortas</t>
   </si>
   <si>
-    <t xml:space="preserve">Esta es una torta de color rosado q sabe rico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta verde</t>
+    <t xml:space="preserve">3 bizcochos de chocolate de 18 cm y 2 rellenos de crema con frutilla. Rinde de 15 a 20 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Choco party</t>
   </si>
   <si>
     <t xml:space="preserve">tortas2.png</t>
   </si>
   <si>
-    <t xml:space="preserve">Esta torta se logra al unir los colores azul y amarillo</t>
+    <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de crema oreo más confituras y drip de chocolate. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Flores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas3.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de dulce de leche con cobertura de ganache de chocolate y forrado en fondat. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Azzurra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas4.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de crema de dulce de leche. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Fiori</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas10.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 bizcochos de chocolate de 14 cm, 1 relleno de dulce de leche más decoración comestible. Rinde de 4 a 6 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Mamá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas5.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de vainilla de 20 cm y 2 rellenos de crema con durazno. Rinde de 20 a 25 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Bianca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas6.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de limón de 14 cm, 2 rellenos de ganache de limón y cobertura de chocolate blanco. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Rosita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas7.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 bizcochos de Red Velvet de 18 cm, 1 relleno de crema con frutilla. Rinde de 8 a 10 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Daddy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas8.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de crema con durazno más decoración personalizada. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Sueño rosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas9.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de chocolate de 20 cm y 2 rellenos de dulce de leche más decoraciones comestibles. Rinde de 20 a 25 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Osita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas11.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de crema Bariloche con cobertura de ganache de chocolate, forrado en fondat y decoración en porcelana fría. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Dulce de leche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas12.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de vainilla de 18 cm y 2 rellenos de crema de dulce de leche. Rinde de 15 a 20 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Yule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas13.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de ganache de chocolate y cobertura de chocolate más decoración personalizada. Rinde de 6 a 8 porciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta Duraznos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortas14.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 bizcochos de vainilla de 20 cm, 1 relleno de crema con duraznos más decoración frutal. Rinde de 12 a 15 porciones.</t>
   </si>
   <si>
     <t xml:space="preserve">Torre gigante</t>
@@ -67,25 +175,7 @@
     <t xml:space="preserve">Regalos</t>
   </si>
   <si>
-    <t xml:space="preserve">Torre que es muy grande</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta flores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas3.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si te gustan las mariposas te gustan las flores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta azul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas4.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Azul es el color del mar, azul es el color de mi capital</t>
+    <t xml:space="preserve">Juego clásico de equilibrio, ideal para compartir en familia</t>
   </si>
   <si>
     <t xml:space="preserve">Juego 5 en 1</t>
@@ -94,34 +184,7 @@
     <t xml:space="preserve">regalo2.png</t>
   </si>
   <si>
-    <t xml:space="preserve">Hay 5 juegos acá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta naranja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas10.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lindas mariposas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta mamá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas5.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si quieres a tu mamá compra esta torta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta roja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas6.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">También es blanca, pero hay q decir q no al racismo</t>
+    <t xml:space="preserve">Cinco juegos clásicos en un solo set para horas de diversión</t>
   </si>
   <si>
     <t xml:space="preserve">Lotería</t>
@@ -130,70 +193,7 @@
     <t xml:space="preserve">regalo3.png</t>
   </si>
   <si>
-    <t xml:space="preserve">Gana o pierde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta rosita</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas7.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Otra más de color rosa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta papá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas8.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trae cerveza incluida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta mariposas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas9.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trae mariposas rosadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta osito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas11.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiene un osito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta dulce de leche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas12.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trae bastante dulce de leche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta choco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas13.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puro sabor choco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Torta duraznos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tortas14.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiene duraznos buenos</t>
+    <t xml:space="preserve">Pon a prueba tu suerte y comparte momentos inolvidables</t>
   </si>
 </sst>
 </file>
@@ -268,7 +268,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -279,6 +279,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -407,10 +411,11 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="57.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="103.23"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -435,7 +440,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1500</v>
+        <v>2700</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -452,7 +457,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2100</v>
+        <v>2500</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>10</v>
@@ -464,258 +469,258 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>990</v>
+        <v>3500</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1900</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>3500</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="2" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>1800</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>3800</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>810</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="2" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>1900</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>2300</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="1" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>3100</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="1" t="n">
+        <v>4100</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>690</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="2" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="1" t="n">
+        <v>5300</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="1" t="n">
-        <v>2100</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="1" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="1" t="n">
-        <v>3400</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="1" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="B15" s="1" t="n">
+        <v>2900</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="0" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="1" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="2" t="n">
+        <v>990</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="0" t="n">
-        <v>3100</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="0" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="B17" s="2" t="n">
+        <v>810</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="D17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="B18" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="D18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimización de imágenes: conversión a AVIF
</commit_message>
<xml_diff>
--- a/public/data/productos.xlsx
+++ b/public/data/productos.xlsx
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Torta Princesa</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas1.png</t>
+    <t xml:space="preserve">tortas1.avif</t>
   </si>
   <si>
     <t xml:space="preserve">Tortas</t>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Torta Choco party</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas2.png</t>
+    <t xml:space="preserve">tortas2.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de crema oreo más confituras y drip de chocolate. Rinde de 6 a 8 porciones.</t>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Torta Flores</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas3.png</t>
+    <t xml:space="preserve">tortas3.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de dulce de leche con cobertura de ganache de chocolate y forrado en fondat. Rinde de 6 a 8 porciones.</t>
@@ -70,7 +70,7 @@
     <t xml:space="preserve">Torta Azzurra</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas4.png</t>
+    <t xml:space="preserve">tortas4.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de crema de dulce de leche. Rinde de 6 a 8 porciones.</t>
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Torta Fiori</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas10.png</t>
+    <t xml:space="preserve">tortas10.avif</t>
   </si>
   <si>
     <t xml:space="preserve">2 bizcochos de chocolate de 14 cm, 1 relleno de dulce de leche más decoración comestible. Rinde de 4 a 6 porciones.</t>
@@ -88,7 +88,7 @@
     <t xml:space="preserve">Torta Mamá</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas5.png</t>
+    <t xml:space="preserve">tortas5.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de vainilla de 20 cm y 2 rellenos de crema con durazno. Rinde de 20 a 25 porciones.</t>
@@ -97,7 +97,7 @@
     <t xml:space="preserve">Torta Bianca</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas6.png</t>
+    <t xml:space="preserve">tortas6.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de limón de 14 cm, 2 rellenos de ganache de limón y cobertura de chocolate blanco. Rinde de 6 a 8 porciones.</t>
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Torta Rosita</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas7.png</t>
+    <t xml:space="preserve">tortas7.avif</t>
   </si>
   <si>
     <t xml:space="preserve">2 bizcochos de Red Velvet de 18 cm, 1 relleno de crema con frutilla. Rinde de 8 a 10 porciones.</t>
@@ -115,7 +115,7 @@
     <t xml:space="preserve">Torta Daddy</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas8.png</t>
+    <t xml:space="preserve">tortas8.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de vainilla de 14 cm, 2 rellenos de crema con durazno más decoración personalizada. Rinde de 6 a 8 porciones.</t>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Torta Sueño rosa</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas9.png</t>
+    <t xml:space="preserve">tortas9.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de chocolate de 20 cm y 2 rellenos de dulce de leche más decoraciones comestibles. Rinde de 20 a 25 porciones.</t>
@@ -133,7 +133,7 @@
     <t xml:space="preserve">Torta Osita</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas11.png</t>
+    <t xml:space="preserve">tortas11.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de crema Bariloche con cobertura de ganache de chocolate, forrado en fondat y decoración en porcelana fría. Rinde de 6 a 8 porciones.</t>
@@ -142,7 +142,7 @@
     <t xml:space="preserve">Torta Dulce de leche</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas12.png</t>
+    <t xml:space="preserve">tortas12.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de vainilla de 18 cm y 2 rellenos de crema de dulce de leche. Rinde de 15 a 20 porciones.</t>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Torta Yule</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas13.png</t>
+    <t xml:space="preserve">tortas13.avif</t>
   </si>
   <si>
     <t xml:space="preserve">3 bizcochos de chocolate de 14 cm, 2 rellenos de ganache de chocolate y cobertura de chocolate más decoración personalizada. Rinde de 6 a 8 porciones.</t>
@@ -160,7 +160,7 @@
     <t xml:space="preserve">Torta Duraznos</t>
   </si>
   <si>
-    <t xml:space="preserve">tortas14.png</t>
+    <t xml:space="preserve">tortas14.avif</t>
   </si>
   <si>
     <t xml:space="preserve">2 bizcochos de vainilla de 20 cm, 1 relleno de crema con duraznos más decoración frutal. Rinde de 12 a 15 porciones.</t>
@@ -169,7 +169,7 @@
     <t xml:space="preserve">Torre gigante</t>
   </si>
   <si>
-    <t xml:space="preserve">regalo1.png</t>
+    <t xml:space="preserve">regalo1.avif</t>
   </si>
   <si>
     <t xml:space="preserve">Regalos</t>
@@ -181,7 +181,7 @@
     <t xml:space="preserve">Juego 5 en 1</t>
   </si>
   <si>
-    <t xml:space="preserve">regalo2.png</t>
+    <t xml:space="preserve">regalo2.avif</t>
   </si>
   <si>
     <t xml:space="preserve">Cinco juegos clásicos en un solo set para horas de diversión</t>
@@ -190,7 +190,7 @@
     <t xml:space="preserve">Lotería</t>
   </si>
   <si>
-    <t xml:space="preserve">regalo3.png</t>
+    <t xml:space="preserve">regalo3.avif</t>
   </si>
   <si>
     <t xml:space="preserve">Pon a prueba tu suerte y comparte momentos inolvidables</t>

</xml_diff>